<commit_message>
Atualizacao mensal automatica (2026-07-19)
</commit_message>
<xml_diff>
--- a/reports/09_credito_detalhado.xlsx
+++ b/reports/09_credito_detalhado.xlsx
@@ -16,10 +16,10 @@
     <sheet name="Nao parseados (auditoria)" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Juros por modalidade'!$A$1:$G$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Juros por modalidade'!$A$1:$G$160</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Inadimplencia por modalidade'!$A$1:$G$180</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Saldo por porte e MEI'!$A$1:$H$370</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ICC e spread'!$A$1:$G$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'ICC e spread'!$A$1:$G$80</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Prazo medio'!$A$1:$G$147</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Concessoes por modalidade'!$A$1:$F$79</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Nao parseados (auditoria)'!$A$1:$C$25</definedName>
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G161"/>
+  <dimension ref="A1:G160"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3845,17 +3845,17 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>Crédito rotativo vinculado a cartão de crédito</t>
+          <t>Adiantamentos a depositantes</t>
         </is>
       </c>
       <c r="E122" t="n">
         <v>202304</v>
       </c>
       <c r="F122" s="1" t="n">
-        <v>272.6</v>
+        <v>224.9</v>
       </c>
       <c r="G122" s="1" t="n">
-        <v>15.17</v>
+        <v>-6.8</v>
       </c>
     </row>
     <row r="123">
@@ -3876,17 +3876,17 @@
       </c>
       <c r="D123" t="inlineStr">
         <is>
-          <t>Adiantamentos a depositantes</t>
+          <t>Conta Garantia</t>
         </is>
       </c>
       <c r="E123" t="n">
         <v>202304</v>
       </c>
       <c r="F123" s="1" t="n">
-        <v>224.9</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="G123" s="1" t="n">
-        <v>-6.8</v>
+        <v>9.16</v>
       </c>
     </row>
     <row r="124">
@@ -3907,17 +3907,17 @@
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>Conta Garantia</t>
+          <t>Cartão de crédito - compra ou fatura parcelada pela instituição financeira emitente do cartão</t>
         </is>
       </c>
       <c r="E124" t="n">
         <v>202304</v>
       </c>
       <c r="F124" s="1" t="n">
-        <v>73.90000000000001</v>
+        <v>54.8</v>
       </c>
       <c r="G124" s="1" t="n">
-        <v>9.16</v>
+        <v>-3.69</v>
       </c>
     </row>
     <row r="125">
@@ -3938,17 +3938,17 @@
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>Cartão de crédito - compra ou fatura parcelada pela instituição financeira emitente do cartão</t>
+          <t>Capital de giro com prazo de vencimento até 365 dias</t>
         </is>
       </c>
       <c r="E125" t="n">
         <v>202304</v>
       </c>
       <c r="F125" s="1" t="n">
-        <v>54.8</v>
+        <v>39.9</v>
       </c>
       <c r="G125" s="1" t="n">
-        <v>-3.69</v>
+        <v>13.03</v>
       </c>
     </row>
     <row r="126">
@@ -3969,17 +3969,17 @@
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>Capital de giro com prazo de vencimento até 365 dias</t>
+          <t>Outros empréstimos</t>
         </is>
       </c>
       <c r="E126" t="n">
         <v>202304</v>
       </c>
       <c r="F126" s="1" t="n">
-        <v>39.9</v>
+        <v>32</v>
       </c>
       <c r="G126" s="1" t="n">
-        <v>13.03</v>
+        <v>-3.9</v>
       </c>
     </row>
     <row r="127">
@@ -4000,17 +4000,17 @@
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>Outros empréstimos</t>
+          <t>Microcrédito</t>
         </is>
       </c>
       <c r="E127" t="n">
         <v>202304</v>
       </c>
       <c r="F127" s="1" t="n">
-        <v>32</v>
+        <v>30.1</v>
       </c>
       <c r="G127" s="1" t="n">
-        <v>-3.9</v>
+        <v>2.03</v>
       </c>
     </row>
     <row r="128">
@@ -4031,17 +4031,17 @@
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>Microcrédito</t>
+          <t>Desconto de duplicatas</t>
         </is>
       </c>
       <c r="E128" t="n">
         <v>202304</v>
       </c>
       <c r="F128" s="1" t="n">
-        <v>30.1</v>
+        <v>29.5</v>
       </c>
       <c r="G128" s="1" t="n">
-        <v>2.03</v>
+        <v>8.06</v>
       </c>
     </row>
     <row r="129">
@@ -4062,17 +4062,17 @@
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>Desconto de duplicatas</t>
+          <t>Desconto de cheques</t>
         </is>
       </c>
       <c r="E129" t="n">
         <v>202304</v>
       </c>
       <c r="F129" s="1" t="n">
-        <v>29.5</v>
+        <v>28.3</v>
       </c>
       <c r="G129" s="1" t="n">
-        <v>8.06</v>
+        <v>8.43</v>
       </c>
     </row>
     <row r="130">
@@ -4093,17 +4093,17 @@
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>Desconto de cheques</t>
+          <t>Outros financiamentos com interveniência</t>
         </is>
       </c>
       <c r="E130" t="n">
         <v>202304</v>
       </c>
       <c r="F130" s="1" t="n">
-        <v>28.3</v>
+        <v>27.4</v>
       </c>
       <c r="G130" s="1" t="n">
-        <v>8.43</v>
+        <v>6.61</v>
       </c>
     </row>
     <row r="131">
@@ -4124,17 +4124,17 @@
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>Outros financiamentos com interveniência</t>
+          <t>Capital de giro com prazo de vencimento superior a 365 dias</t>
         </is>
       </c>
       <c r="E131" t="n">
         <v>202304</v>
       </c>
       <c r="F131" s="1" t="n">
-        <v>27.4</v>
+        <v>26.4</v>
       </c>
       <c r="G131" s="1" t="n">
-        <v>6.61</v>
+        <v>14.29</v>
       </c>
     </row>
     <row r="132">
@@ -4155,7 +4155,7 @@
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>Capital de giro com prazo de vencimento superior a 365 dias</t>
+          <t>Outros títulos descontados</t>
         </is>
       </c>
       <c r="E132" t="n">
@@ -4165,7 +4165,7 @@
         <v>26.4</v>
       </c>
       <c r="G132" s="1" t="n">
-        <v>14.29</v>
+        <v>3.94</v>
       </c>
     </row>
     <row r="133">
@@ -4186,17 +4186,17 @@
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>Outros títulos descontados</t>
+          <t>Outros direitos creditórios descontados</t>
         </is>
       </c>
       <c r="E133" t="n">
         <v>202304</v>
       </c>
       <c r="F133" s="1" t="n">
-        <v>26.4</v>
+        <v>25.6</v>
       </c>
       <c r="G133" s="1" t="n">
-        <v>3.94</v>
+        <v>11.79</v>
       </c>
     </row>
     <row r="134">
@@ -4217,17 +4217,17 @@
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>Outros direitos creditórios descontados</t>
+          <t>Antecipação de fatura de cartão de crédito</t>
         </is>
       </c>
       <c r="E134" t="n">
         <v>202304</v>
       </c>
       <c r="F134" s="1" t="n">
-        <v>25.6</v>
+        <v>25.3</v>
       </c>
       <c r="G134" s="1" t="n">
-        <v>11.79</v>
+        <v>13.96</v>
       </c>
     </row>
     <row r="135">
@@ -4248,17 +4248,17 @@
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>Antecipação de fatura de cartão de crédito</t>
+          <t>Outros financiamentos</t>
         </is>
       </c>
       <c r="E135" t="n">
         <v>202304</v>
       </c>
       <c r="F135" s="1" t="n">
-        <v>25.3</v>
+        <v>21.7</v>
       </c>
       <c r="G135" s="1" t="n">
-        <v>13.96</v>
+        <v>29.94</v>
       </c>
     </row>
     <row r="136">
@@ -4279,17 +4279,17 @@
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>Outros financiamentos</t>
+          <t>Arrendamento financeiro de veículos automotores até 2 toneladas</t>
         </is>
       </c>
       <c r="E136" t="n">
         <v>202304</v>
       </c>
       <c r="F136" s="1" t="n">
-        <v>21.7</v>
+        <v>19.6</v>
       </c>
       <c r="G136" s="1" t="n">
-        <v>29.94</v>
+        <v>0.51</v>
       </c>
     </row>
     <row r="137">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>Arrendamento financeiro de veículos automotores até 2 toneladas</t>
+          <t>Home Equity</t>
         </is>
       </c>
       <c r="E137" t="n">
@@ -4320,7 +4320,7 @@
         <v>19.6</v>
       </c>
       <c r="G137" s="1" t="n">
-        <v>0.51</v>
+        <v>106.32</v>
       </c>
     </row>
     <row r="138">
@@ -4341,17 +4341,17 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>Home Equity</t>
+          <t>Aquisição de bens - outros bens</t>
         </is>
       </c>
       <c r="E138" t="n">
         <v>202304</v>
       </c>
       <c r="F138" s="1" t="n">
-        <v>19.6</v>
+        <v>18.9</v>
       </c>
       <c r="G138" s="1" t="n">
-        <v>106.32</v>
+        <v>11.18</v>
       </c>
     </row>
     <row r="139">
@@ -4372,17 +4372,17 @@
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>Aquisição de bens - outros bens</t>
+          <t>Aquisição de bens - veículos automotores</t>
         </is>
       </c>
       <c r="E139" t="n">
         <v>202304</v>
       </c>
       <c r="F139" s="1" t="n">
-        <v>18.9</v>
+        <v>17.9</v>
       </c>
       <c r="G139" s="1" t="n">
-        <v>11.18</v>
+        <v>13.29</v>
       </c>
     </row>
     <row r="140">
@@ -4403,17 +4403,17 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>Aquisição de bens - veículos automotores</t>
+          <t>Recebíveis adquiridos</t>
         </is>
       </c>
       <c r="E140" t="n">
         <v>202304</v>
       </c>
       <c r="F140" s="1" t="n">
-        <v>17.9</v>
+        <v>17.1</v>
       </c>
       <c r="G140" s="1" t="n">
-        <v>13.29</v>
+        <v>-8.56</v>
       </c>
     </row>
     <row r="141">
@@ -4434,17 +4434,17 @@
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>Recebíveis adquiridos</t>
+          <t>Vendor</t>
         </is>
       </c>
       <c r="E141" t="n">
         <v>202304</v>
       </c>
       <c r="F141" s="1" t="n">
-        <v>17.1</v>
+        <v>17</v>
       </c>
       <c r="G141" s="1" t="n">
-        <v>-8.56</v>
+        <v>17.24</v>
       </c>
     </row>
     <row r="142">
@@ -4465,17 +4465,17 @@
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>Vendor</t>
+          <t>Compror</t>
         </is>
       </c>
       <c r="E142" t="n">
         <v>202304</v>
       </c>
       <c r="F142" s="1" t="n">
-        <v>17</v>
+        <v>16.7</v>
       </c>
       <c r="G142" s="1" t="n">
-        <v>17.24</v>
+        <v>-9.24</v>
       </c>
     </row>
     <row r="143">
@@ -4496,17 +4496,17 @@
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>Compror</t>
+          <t>Financiamento à exportação</t>
         </is>
       </c>
       <c r="E143" t="n">
         <v>202304</v>
       </c>
       <c r="F143" s="1" t="n">
-        <v>16.7</v>
+        <v>15.9</v>
       </c>
       <c r="G143" s="1" t="n">
-        <v>-9.24</v>
+        <v>-19.7</v>
       </c>
     </row>
     <row r="144">
@@ -4527,17 +4527,17 @@
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>Financiamento à exportação</t>
+          <t>Arrendamento financeiro</t>
         </is>
       </c>
       <c r="E144" t="n">
         <v>202304</v>
       </c>
       <c r="F144" s="1" t="n">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
       <c r="G144" s="1" t="n">
-        <v>-19.7</v>
+        <v>8.970000000000001</v>
       </c>
     </row>
     <row r="145">
@@ -4558,17 +4558,17 @@
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>Arrendamento financeiro</t>
+          <t>Financiamento de projeto</t>
         </is>
       </c>
       <c r="E145" t="n">
         <v>202304</v>
       </c>
       <c r="F145" s="1" t="n">
-        <v>15.8</v>
+        <v>14.9</v>
       </c>
       <c r="G145" s="1" t="n">
-        <v>8.970000000000001</v>
+        <v>39.25</v>
       </c>
     </row>
     <row r="146">
@@ -4589,17 +4589,17 @@
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>Financiamento de projeto</t>
+          <t>Financiamento rural - comercialização</t>
         </is>
       </c>
       <c r="E146" t="n">
         <v>202304</v>
       </c>
       <c r="F146" s="1" t="n">
-        <v>14.9</v>
+        <v>14.5</v>
       </c>
       <c r="G146" s="1" t="n">
-        <v>39.25</v>
+        <v>19.83</v>
       </c>
     </row>
     <row r="147">
@@ -4620,17 +4620,17 @@
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>Financiamento rural - comercialização</t>
+          <t>Financiamento rural - custeio</t>
         </is>
       </c>
       <c r="E147" t="n">
         <v>202304</v>
       </c>
       <c r="F147" s="1" t="n">
-        <v>14.5</v>
+        <v>13.9</v>
       </c>
       <c r="G147" s="1" t="n">
-        <v>19.83</v>
+        <v>15.83</v>
       </c>
     </row>
     <row r="148">
@@ -4651,17 +4651,17 @@
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>Financiamento rural - custeio</t>
+          <t>Avais e fianças honrados</t>
         </is>
       </c>
       <c r="E148" t="n">
         <v>202304</v>
       </c>
       <c r="F148" s="1" t="n">
-        <v>13.9</v>
+        <v>12.9</v>
       </c>
       <c r="G148" s="1" t="n">
-        <v>15.83</v>
+        <v>44.94</v>
       </c>
     </row>
     <row r="149">
@@ -4682,17 +4682,17 @@
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>Avais e fianças honrados</t>
+          <t>Títulos e créditos a receber</t>
         </is>
       </c>
       <c r="E149" t="n">
         <v>202304</v>
       </c>
       <c r="F149" s="1" t="n">
-        <v>12.9</v>
+        <v>12.4</v>
       </c>
       <c r="G149" s="1" t="n">
-        <v>44.94</v>
+        <v>-31.87</v>
       </c>
     </row>
     <row r="150">
@@ -4713,17 +4713,17 @@
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>Títulos e créditos a receber</t>
+          <t>Financiamento rural - investimento</t>
         </is>
       </c>
       <c r="E150" t="n">
         <v>202304</v>
       </c>
       <c r="F150" s="1" t="n">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="G150" s="1" t="n">
-        <v>-31.87</v>
+        <v>33.7</v>
       </c>
     </row>
     <row r="151">
@@ -4744,17 +4744,17 @@
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>Financiamento rural - investimento</t>
+          <t>Financiamento imobiliário - empreendim, exceto habitac.</t>
         </is>
       </c>
       <c r="E151" t="n">
         <v>202304</v>
       </c>
       <c r="F151" s="1" t="n">
-        <v>12.3</v>
+        <v>11</v>
       </c>
       <c r="G151" s="1" t="n">
-        <v>33.7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="152">
@@ -4775,17 +4775,17 @@
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>Financiamento imobiliário - empreendim, exceto habitac.</t>
+          <t>Financiamento habitacional - carteira hipotecária</t>
         </is>
       </c>
       <c r="E152" t="n">
         <v>202304</v>
       </c>
       <c r="F152" s="1" t="n">
-        <v>11</v>
+        <v>10.7</v>
       </c>
       <c r="G152" s="1" t="n">
-        <v>10</v>
+        <v>245.16</v>
       </c>
     </row>
     <row r="153">
@@ -4806,17 +4806,17 @@
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>Financiamento habitacional - carteira hipotecária</t>
+          <t>Financiamento à importação</t>
         </is>
       </c>
       <c r="E153" t="n">
         <v>202304</v>
       </c>
       <c r="F153" s="1" t="n">
-        <v>10.7</v>
+        <v>10.1</v>
       </c>
       <c r="G153" s="1" t="n">
-        <v>245.16</v>
+        <v>98.04000000000001</v>
       </c>
     </row>
     <row r="154">
@@ -4837,17 +4837,17 @@
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>Financiamento à importação</t>
+          <t>Adiantamento sobre cambiais entregues</t>
         </is>
       </c>
       <c r="E154" t="n">
         <v>202304</v>
       </c>
       <c r="F154" s="1" t="n">
-        <v>10.1</v>
+        <v>10</v>
       </c>
       <c r="G154" s="1" t="n">
-        <v>98.04000000000001</v>
+        <v>36.99</v>
       </c>
     </row>
     <row r="155">
@@ -4868,17 +4868,17 @@
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>Adiantamento sobre cambiais entregues</t>
+          <t>Adiantamento sobre contratos de câmbio</t>
         </is>
       </c>
       <c r="E155" t="n">
         <v>202304</v>
       </c>
       <c r="F155" s="1" t="n">
-        <v>10</v>
+        <v>9.800000000000001</v>
       </c>
       <c r="G155" s="1" t="n">
-        <v>36.99</v>
+        <v>66.09999999999999</v>
       </c>
     </row>
     <row r="156">
@@ -4899,17 +4899,17 @@
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>Adiantamento sobre contratos de câmbio</t>
+          <t>Arrendamento operacional</t>
         </is>
       </c>
       <c r="E156" t="n">
         <v>202304</v>
       </c>
       <c r="F156" s="1" t="n">
-        <v>9.800000000000001</v>
+        <v>6.5</v>
       </c>
       <c r="G156" s="1" t="n">
-        <v>66.09999999999999</v>
+        <v>-7.14</v>
       </c>
     </row>
     <row r="157">
@@ -4930,17 +4930,17 @@
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>Arrendamento operacional</t>
+          <t>Outros financiamentos à exportação</t>
         </is>
       </c>
       <c r="E157" t="n">
         <v>202304</v>
       </c>
       <c r="F157" s="1" t="n">
-        <v>6.5</v>
+        <v>5</v>
       </c>
       <c r="G157" s="1" t="n">
-        <v>-7.14</v>
+        <v>-75.25</v>
       </c>
     </row>
     <row r="158">
@@ -4961,17 +4961,17 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>Outros financiamentos à exportação</t>
+          <t>Outros com característica de crédito</t>
         </is>
       </c>
       <c r="E158" t="n">
         <v>202304</v>
       </c>
       <c r="F158" s="1" t="n">
-        <v>5</v>
+        <v>3.6</v>
       </c>
       <c r="G158" s="1" t="n">
-        <v>-75.25</v>
+        <v>-43.75</v>
       </c>
     </row>
     <row r="159">
@@ -4992,17 +4992,17 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>Outros com característica de crédito</t>
+          <t>Devedores por compra de valores e bens</t>
         </is>
       </c>
       <c r="E159" t="n">
         <v>202304</v>
       </c>
       <c r="F159" s="1" t="n">
-        <v>3.6</v>
+        <v>2.8</v>
       </c>
       <c r="G159" s="1" t="n">
-        <v>-43.75</v>
+        <v>-3.45</v>
       </c>
     </row>
     <row r="160">
@@ -5023,52 +5023,21 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>Devedores por compra de valores e bens</t>
+          <t>Financiamento de TVM</t>
         </is>
       </c>
       <c r="E160" t="n">
         <v>202304</v>
       </c>
       <c r="F160" s="1" t="n">
-        <v>2.8</v>
+        <v>0</v>
       </c>
       <c r="G160" s="1" t="n">
-        <v>-3.45</v>
-      </c>
-    </row>
-    <row r="161">
-      <c r="A161" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="B161" t="inlineStr">
-        <is>
-          <t>PEQUENO</t>
-        </is>
-      </c>
-      <c r="C161" t="inlineStr">
-        <is>
-          <t>LIVRE</t>
-        </is>
-      </c>
-      <c r="D161" t="inlineStr">
-        <is>
-          <t>Financiamento de TVM</t>
-        </is>
-      </c>
-      <c r="E161" t="n">
-        <v>202304</v>
-      </c>
-      <c r="F161" s="1" t="n">
-        <v>0</v>
-      </c>
-      <c r="G161" s="1" t="n">
         <v>-100</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G161"/>
+  <autoFilter ref="A1:G160"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -20720,7 +20689,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G81"/>
+  <dimension ref="A1:G80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -21504,19 +21473,15 @@
           <t>LIVRE</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr">
-        <is>
-          <t>Crédito pessoal não consignado vinculado à composição de dívidas</t>
-        </is>
-      </c>
+      <c r="D27" t="inlineStr"/>
       <c r="E27" t="n">
         <v>202605</v>
       </c>
       <c r="F27" s="1" t="n">
-        <v>45.88</v>
+        <v>45.41</v>
       </c>
       <c r="G27" s="1" t="n">
-        <v>5.33</v>
+        <v>6.42</v>
       </c>
     </row>
     <row r="28">
@@ -21535,15 +21500,19 @@
           <t>LIVRE</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Cartão de crédito total</t>
+        </is>
+      </c>
       <c r="E28" t="n">
         <v>202605</v>
       </c>
       <c r="F28" s="1" t="n">
-        <v>45.41</v>
+        <v>43.72</v>
       </c>
       <c r="G28" s="1" t="n">
-        <v>6.42</v>
+        <v>3.95</v>
       </c>
     </row>
     <row r="29">
@@ -21564,17 +21533,17 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Cartão de crédito total</t>
+          <t>Crédito não rotativo - Total</t>
         </is>
       </c>
       <c r="E29" t="n">
         <v>202605</v>
       </c>
       <c r="F29" s="1" t="n">
-        <v>43.72</v>
+        <v>43.54</v>
       </c>
       <c r="G29" s="1" t="n">
-        <v>3.95</v>
+        <v>2.04</v>
       </c>
     </row>
     <row r="30">
@@ -21595,17 +21564,17 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Crédito não rotativo - Total</t>
+          <t>Crédito pessoal consignado total</t>
         </is>
       </c>
       <c r="E30" t="n">
         <v>202605</v>
       </c>
       <c r="F30" s="1" t="n">
-        <v>43.54</v>
+        <v>27.14</v>
       </c>
       <c r="G30" s="1" t="n">
-        <v>2.04</v>
+        <v>13.22</v>
       </c>
     </row>
     <row r="31">
@@ -21626,17 +21595,17 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Crédito pessoal consignado total</t>
+          <t>Aquisição de veículos</t>
         </is>
       </c>
       <c r="E31" t="n">
         <v>202605</v>
       </c>
       <c r="F31" s="1" t="n">
-        <v>27.14</v>
+        <v>26.95</v>
       </c>
       <c r="G31" s="1" t="n">
-        <v>13.22</v>
+        <v>0.6</v>
       </c>
     </row>
     <row r="32">
@@ -21657,17 +21626,17 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Aquisição de veículos</t>
+          <t>Crédito pessoal consignado para aposentados e pensionistas do INSS</t>
         </is>
       </c>
       <c r="E32" t="n">
         <v>202605</v>
       </c>
       <c r="F32" s="1" t="n">
-        <v>26.95</v>
+        <v>23.51</v>
       </c>
       <c r="G32" s="1" t="n">
-        <v>0.6</v>
+        <v>1.56</v>
       </c>
     </row>
     <row r="33">
@@ -21688,17 +21657,17 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Crédito pessoal consignado para aposentados e pensionistas do INSS</t>
+          <t>Crédito pessoal consignado para trabalhadores do setor público</t>
         </is>
       </c>
       <c r="E33" t="n">
         <v>202605</v>
       </c>
       <c r="F33" s="1" t="n">
-        <v>23.51</v>
+        <v>23.01</v>
       </c>
       <c r="G33" s="1" t="n">
-        <v>1.56</v>
+        <v>2.36</v>
       </c>
     </row>
     <row r="34">
@@ -21719,17 +21688,17 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Crédito pessoal consignado para trabalhadores do setor público</t>
+          <t>Arrendamento mercantil de veículos</t>
         </is>
       </c>
       <c r="E34" t="n">
         <v>202605</v>
       </c>
       <c r="F34" s="1" t="n">
-        <v>23.01</v>
+        <v>22.24</v>
       </c>
       <c r="G34" s="1" t="n">
-        <v>2.36</v>
+        <v>-4.63</v>
       </c>
     </row>
     <row r="35">
@@ -21750,17 +21719,17 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Arrendamento mercantil de veículos</t>
+          <t>Arrendamento mercantil de outros bens</t>
         </is>
       </c>
       <c r="E35" t="n">
         <v>202605</v>
       </c>
       <c r="F35" s="1" t="n">
-        <v>22.24</v>
+        <v>17.17</v>
       </c>
       <c r="G35" s="1" t="n">
-        <v>-4.63</v>
+        <v>4.63</v>
       </c>
     </row>
     <row r="36">
@@ -21771,27 +21740,19 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>LIVRE</t>
-        </is>
-      </c>
-      <c r="D36" t="inlineStr">
-        <is>
-          <t>Arrendamento mercantil de outros bens</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr"/>
+      <c r="D36" t="inlineStr"/>
       <c r="E36" t="n">
         <v>202605</v>
       </c>
       <c r="F36" s="1" t="n">
-        <v>17.17</v>
+        <v>17.57</v>
       </c>
       <c r="G36" s="1" t="n">
-        <v>4.63</v>
+        <v>3.47</v>
       </c>
     </row>
     <row r="37">
@@ -21806,7 +21767,11 @@
         </is>
       </c>
       <c r="C37" t="inlineStr"/>
-      <c r="D37" t="inlineStr"/>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>Crédito não rotativo - Total</t>
+        </is>
+      </c>
       <c r="E37" t="n">
         <v>202605</v>
       </c>
@@ -21828,20 +21793,24 @@
           <t>PJ</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr"/>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>DIRECIONADO</t>
+        </is>
+      </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Crédito não rotativo - Total</t>
+          <t>Crédito rural com taxas de mercado</t>
         </is>
       </c>
       <c r="E38" t="n">
         <v>202605</v>
       </c>
       <c r="F38" s="1" t="n">
-        <v>17.57</v>
+        <v>13.56</v>
       </c>
       <c r="G38" s="1" t="n">
-        <v>3.47</v>
+        <v>2.19</v>
       </c>
     </row>
     <row r="39">
@@ -21862,17 +21831,17 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Crédito rural com taxas de mercado</t>
+          <t>Crédito rural total</t>
         </is>
       </c>
       <c r="E39" t="n">
         <v>202605</v>
       </c>
       <c r="F39" s="1" t="n">
-        <v>13.56</v>
+        <v>13.09</v>
       </c>
       <c r="G39" s="1" t="n">
-        <v>2.19</v>
+        <v>4.39</v>
       </c>
     </row>
     <row r="40">
@@ -21893,17 +21862,17 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Crédito rural total</t>
+          <t>Crédito rural com taxas reguladas</t>
         </is>
       </c>
       <c r="E40" t="n">
         <v>202605</v>
       </c>
       <c r="F40" s="1" t="n">
-        <v>13.09</v>
+        <v>12.18</v>
       </c>
       <c r="G40" s="1" t="n">
-        <v>4.39</v>
+        <v>5.64</v>
       </c>
     </row>
     <row r="41">
@@ -21924,17 +21893,17 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Crédito rural com taxas reguladas</t>
+          <t>Capital de giro com recursos do BNDES</t>
         </is>
       </c>
       <c r="E41" t="n">
         <v>202605</v>
       </c>
       <c r="F41" s="1" t="n">
-        <v>12.18</v>
+        <v>11.93</v>
       </c>
       <c r="G41" s="1" t="n">
-        <v>5.64</v>
+        <v>-1.16</v>
       </c>
     </row>
     <row r="42">
@@ -21953,19 +21922,15 @@
           <t>DIRECIONADO</t>
         </is>
       </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>Capital de giro com recursos do BNDES</t>
-        </is>
-      </c>
+      <c r="D42" t="inlineStr"/>
       <c r="E42" t="n">
         <v>202605</v>
       </c>
       <c r="F42" s="1" t="n">
-        <v>11.93</v>
+        <v>11.35</v>
       </c>
       <c r="G42" s="1" t="n">
-        <v>-1.16</v>
+        <v>7.18</v>
       </c>
     </row>
     <row r="43">
@@ -21984,15 +21949,19 @@
           <t>DIRECIONADO</t>
         </is>
       </c>
-      <c r="D43" t="inlineStr"/>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>Financiamento imobiliário com taxas de mercado</t>
+        </is>
+      </c>
       <c r="E43" t="n">
         <v>202605</v>
       </c>
       <c r="F43" s="1" t="n">
-        <v>11.35</v>
+        <v>10.91</v>
       </c>
       <c r="G43" s="1" t="n">
-        <v>7.18</v>
+        <v>3.31</v>
       </c>
     </row>
     <row r="44">
@@ -22013,17 +21982,17 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Financiamento imobiliário com taxas de mercado</t>
+          <t>Financiamento imobiliário total</t>
         </is>
       </c>
       <c r="E44" t="n">
         <v>202605</v>
       </c>
       <c r="F44" s="1" t="n">
-        <v>10.91</v>
+        <v>10.85</v>
       </c>
       <c r="G44" s="1" t="n">
-        <v>3.31</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="45">
@@ -22044,17 +22013,17 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Financiamento imobiliário total</t>
+          <t>Financiamento imobiliário com taxas reguladas</t>
         </is>
       </c>
       <c r="E45" t="n">
         <v>202605</v>
       </c>
       <c r="F45" s="1" t="n">
-        <v>10.85</v>
+        <v>10.66</v>
       </c>
       <c r="G45" s="1" t="n">
-        <v>2.75</v>
+        <v>0.95</v>
       </c>
     </row>
     <row r="46">
@@ -22075,17 +22044,17 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Financiamento imobiliário com taxas reguladas</t>
+          <t>Financiamento de investimentos com recursos do BNDES</t>
         </is>
       </c>
       <c r="E46" t="n">
         <v>202605</v>
       </c>
       <c r="F46" s="1" t="n">
-        <v>10.66</v>
+        <v>10.35</v>
       </c>
       <c r="G46" s="1" t="n">
-        <v>0.95</v>
+        <v>6.92</v>
       </c>
     </row>
     <row r="47">
@@ -22106,17 +22075,17 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Financiamento de investimentos com recursos do BNDES</t>
+          <t>Financiamento agroindustrial com recursos do BNDES</t>
         </is>
       </c>
       <c r="E47" t="n">
         <v>202605</v>
       </c>
       <c r="F47" s="1" t="n">
-        <v>10.35</v>
+        <v>9.33</v>
       </c>
       <c r="G47" s="1" t="n">
-        <v>6.92</v>
+        <v>6.39</v>
       </c>
     </row>
     <row r="48">
@@ -22132,22 +22101,22 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DIRECIONADO</t>
+          <t>LIVRE</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Financiamento agroindustrial com recursos do BNDES</t>
+          <t>Cheque especial</t>
         </is>
       </c>
       <c r="E48" t="n">
         <v>202605</v>
       </c>
       <c r="F48" s="1" t="n">
-        <v>9.33</v>
+        <v>360.84</v>
       </c>
       <c r="G48" s="1" t="n">
-        <v>6.39</v>
+        <v>1.09</v>
       </c>
     </row>
     <row r="49">
@@ -22168,17 +22137,17 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Cheque especial</t>
+          <t>Cartão de crédito rotativo</t>
         </is>
       </c>
       <c r="E49" t="n">
         <v>202605</v>
       </c>
       <c r="F49" s="1" t="n">
-        <v>360.84</v>
+        <v>250.32</v>
       </c>
       <c r="G49" s="1" t="n">
-        <v>1.09</v>
+        <v>6.85</v>
       </c>
     </row>
     <row r="50">
@@ -22199,17 +22168,17 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Cartão de crédito rotativo</t>
+          <t>Cartão de crédito parcelado</t>
         </is>
       </c>
       <c r="E50" t="n">
         <v>202605</v>
       </c>
       <c r="F50" s="1" t="n">
-        <v>250.32</v>
+        <v>148.45</v>
       </c>
       <c r="G50" s="1" t="n">
-        <v>6.85</v>
+        <v>6.77</v>
       </c>
     </row>
     <row r="51">
@@ -22230,17 +22199,17 @@
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Cartão de crédito parcelado</t>
+          <t>Conta garantida</t>
         </is>
       </c>
       <c r="E51" t="n">
         <v>202605</v>
       </c>
       <c r="F51" s="1" t="n">
-        <v>148.45</v>
+        <v>63.5</v>
       </c>
       <c r="G51" s="1" t="n">
-        <v>6.77</v>
+        <v>9.99</v>
       </c>
     </row>
     <row r="52">
@@ -22261,17 +22230,17 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Conta garantida</t>
+          <t>Capital de giro rotativo</t>
         </is>
       </c>
       <c r="E52" t="n">
         <v>202605</v>
       </c>
       <c r="F52" s="1" t="n">
-        <v>63.5</v>
+        <v>33.32</v>
       </c>
       <c r="G52" s="1" t="n">
-        <v>9.99</v>
+        <v>10.15</v>
       </c>
     </row>
     <row r="53">
@@ -22292,17 +22261,17 @@
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Capital de giro rotativo</t>
+          <t>Desconto de cheques</t>
         </is>
       </c>
       <c r="E53" t="n">
         <v>202605</v>
       </c>
       <c r="F53" s="1" t="n">
-        <v>33.32</v>
+        <v>32.75</v>
       </c>
       <c r="G53" s="1" t="n">
-        <v>10.15</v>
+        <v>-14.74</v>
       </c>
     </row>
     <row r="54">
@@ -22323,17 +22292,17 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Desconto de cheques</t>
+          <t>Cartão de crédito total</t>
         </is>
       </c>
       <c r="E54" t="n">
         <v>202605</v>
       </c>
       <c r="F54" s="1" t="n">
-        <v>32.75</v>
+        <v>26.75</v>
       </c>
       <c r="G54" s="1" t="n">
-        <v>-14.74</v>
+        <v>16.61</v>
       </c>
     </row>
     <row r="55">
@@ -22354,17 +22323,17 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Cartão de crédito total</t>
+          <t>Capital de giro com prazo de até 365 dias</t>
         </is>
       </c>
       <c r="E55" t="n">
         <v>202605</v>
       </c>
       <c r="F55" s="1" t="n">
-        <v>26.75</v>
+        <v>25.21</v>
       </c>
       <c r="G55" s="1" t="n">
-        <v>16.61</v>
+        <v>8.85</v>
       </c>
     </row>
     <row r="56">
@@ -22385,17 +22354,17 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Capital de giro com prazo de até 365 dias</t>
+          <t>Capital de giro total</t>
         </is>
       </c>
       <c r="E56" t="n">
         <v>202605</v>
       </c>
       <c r="F56" s="1" t="n">
-        <v>25.21</v>
+        <v>22.93</v>
       </c>
       <c r="G56" s="1" t="n">
-        <v>8.85</v>
+        <v>4.94</v>
       </c>
     </row>
     <row r="57">
@@ -22414,19 +22383,15 @@
           <t>LIVRE</t>
         </is>
       </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>Capital de giro total</t>
-        </is>
-      </c>
+      <c r="D57" t="inlineStr"/>
       <c r="E57" t="n">
         <v>202605</v>
       </c>
       <c r="F57" s="1" t="n">
-        <v>22.93</v>
+        <v>22.11</v>
       </c>
       <c r="G57" s="1" t="n">
-        <v>4.94</v>
+        <v>5.69</v>
       </c>
     </row>
     <row r="58">
@@ -22445,7 +22410,11 @@
           <t>LIVRE</t>
         </is>
       </c>
-      <c r="D58" t="inlineStr"/>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>Crédito não rotativo - Total</t>
+        </is>
+      </c>
       <c r="E58" t="n">
         <v>202605</v>
       </c>
@@ -22474,17 +22443,17 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Crédito não rotativo - Total</t>
+          <t>Capital de giro com prazo superior a 365 dias</t>
         </is>
       </c>
       <c r="E59" t="n">
         <v>202605</v>
       </c>
       <c r="F59" s="1" t="n">
-        <v>22.11</v>
+        <v>22.08</v>
       </c>
       <c r="G59" s="1" t="n">
-        <v>5.69</v>
+        <v>3.56</v>
       </c>
     </row>
     <row r="60">
@@ -22505,17 +22474,17 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Capital de giro com prazo superior a 365 dias</t>
+          <t>Aquisição de outros bens</t>
         </is>
       </c>
       <c r="E60" t="n">
         <v>202605</v>
       </c>
       <c r="F60" s="1" t="n">
-        <v>22.08</v>
+        <v>19.13</v>
       </c>
       <c r="G60" s="1" t="n">
-        <v>3.56</v>
+        <v>0.05</v>
       </c>
     </row>
     <row r="61">
@@ -22536,17 +22505,17 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Aquisição de outros bens</t>
+          <t>Desconto de duplicatas e recebíveis</t>
         </is>
       </c>
       <c r="E61" t="n">
         <v>202605</v>
       </c>
       <c r="F61" s="1" t="n">
-        <v>19.13</v>
+        <v>19.07</v>
       </c>
       <c r="G61" s="1" t="n">
-        <v>0.05</v>
+        <v>2.75</v>
       </c>
     </row>
     <row r="62">
@@ -22567,17 +22536,17 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Desconto de duplicatas e recebíveis</t>
+          <t>Vendor</t>
         </is>
       </c>
       <c r="E62" t="n">
         <v>202605</v>
       </c>
       <c r="F62" s="1" t="n">
-        <v>19.07</v>
+        <v>18.48</v>
       </c>
       <c r="G62" s="1" t="n">
-        <v>2.75</v>
+        <v>12.89</v>
       </c>
     </row>
     <row r="63">
@@ -22598,17 +22567,17 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Vendor</t>
+          <t>Aquisição de veículos</t>
         </is>
       </c>
       <c r="E63" t="n">
         <v>202605</v>
       </c>
       <c r="F63" s="1" t="n">
-        <v>18.48</v>
+        <v>18.16</v>
       </c>
       <c r="G63" s="1" t="n">
-        <v>12.89</v>
+        <v>2.95</v>
       </c>
     </row>
     <row r="64">
@@ -22629,17 +22598,17 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>Aquisição de veículos</t>
+          <t>Arrendamento mercantil de veículos</t>
         </is>
       </c>
       <c r="E64" t="n">
         <v>202605</v>
       </c>
       <c r="F64" s="1" t="n">
-        <v>18.16</v>
+        <v>17.51</v>
       </c>
       <c r="G64" s="1" t="n">
-        <v>2.95</v>
+        <v>3.98</v>
       </c>
     </row>
     <row r="65">
@@ -22660,17 +22629,17 @@
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Arrendamento mercantil de veículos</t>
+          <t>Compror</t>
         </is>
       </c>
       <c r="E65" t="n">
         <v>202605</v>
       </c>
       <c r="F65" s="1" t="n">
-        <v>17.51</v>
+        <v>16.97</v>
       </c>
       <c r="G65" s="1" t="n">
-        <v>3.98</v>
+        <v>-7.47</v>
       </c>
     </row>
     <row r="66">
@@ -22691,17 +22660,17 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Compror</t>
+          <t>Antecipação de faturas de cartão</t>
         </is>
       </c>
       <c r="E66" t="n">
         <v>202605</v>
       </c>
       <c r="F66" s="1" t="n">
-        <v>16.97</v>
+        <v>16.55</v>
       </c>
       <c r="G66" s="1" t="n">
-        <v>-7.47</v>
+        <v>-1.02</v>
       </c>
     </row>
     <row r="67">
@@ -22722,17 +22691,17 @@
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Antecipação de faturas de cartão</t>
+          <t>Arrendamento mercantil de outros bens</t>
         </is>
       </c>
       <c r="E67" t="n">
         <v>202605</v>
       </c>
       <c r="F67" s="1" t="n">
-        <v>16.55</v>
+        <v>16.47</v>
       </c>
       <c r="G67" s="1" t="n">
-        <v>-1.02</v>
+        <v>4.37</v>
       </c>
     </row>
     <row r="68">
@@ -22753,17 +22722,17 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Arrendamento mercantil de outros bens</t>
+          <t>Financiamento a exportações</t>
         </is>
       </c>
       <c r="E68" t="n">
         <v>202605</v>
       </c>
       <c r="F68" s="1" t="n">
-        <v>16.47</v>
+        <v>14.18</v>
       </c>
       <c r="G68" s="1" t="n">
-        <v>4.37</v>
+        <v>1.36</v>
       </c>
     </row>
     <row r="69">
@@ -22784,17 +22753,17 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Financiamento a exportações</t>
+          <t>Financiamento a importações</t>
         </is>
       </c>
       <c r="E69" t="n">
         <v>202605</v>
       </c>
       <c r="F69" s="1" t="n">
-        <v>14.18</v>
+        <v>11.98</v>
       </c>
       <c r="G69" s="1" t="n">
-        <v>1.36</v>
+        <v>19.32</v>
       </c>
     </row>
     <row r="70">
@@ -22815,17 +22784,17 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Financiamento a importações</t>
+          <t>Repasse externo</t>
         </is>
       </c>
       <c r="E70" t="n">
         <v>202605</v>
       </c>
       <c r="F70" s="1" t="n">
-        <v>11.98</v>
+        <v>11.82</v>
       </c>
       <c r="G70" s="1" t="n">
-        <v>19.32</v>
+        <v>1.37</v>
       </c>
     </row>
     <row r="71">
@@ -22846,48 +22815,36 @@
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Repasse externo</t>
+          <t>Adiantamentos sobre contratos de câmbio (ACC)</t>
         </is>
       </c>
       <c r="E71" t="n">
         <v>202605</v>
       </c>
       <c r="F71" s="1" t="n">
-        <v>11.82</v>
+        <v>5.75</v>
       </c>
       <c r="G71" s="1" t="n">
-        <v>1.37</v>
+        <v>-7.41</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>ICC</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>LIVRE</t>
-        </is>
-      </c>
-      <c r="D72" t="inlineStr">
-        <is>
-          <t>Adiantamentos sobre contratos de câmbio (ACC)</t>
-        </is>
-      </c>
+          <t>SPREAD_ICC</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
+      <c r="D72" t="inlineStr"/>
       <c r="E72" t="n">
         <v>202605</v>
       </c>
       <c r="F72" s="1" t="n">
-        <v>5.75</v>
+        <v>15.31</v>
       </c>
       <c r="G72" s="1" t="n">
-        <v>-7.41</v>
+        <v>6.62</v>
       </c>
     </row>
     <row r="73">
@@ -22897,16 +22854,20 @@
         </is>
       </c>
       <c r="B73" t="inlineStr"/>
-      <c r="C73" t="inlineStr"/>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>DIRECIONADO</t>
+        </is>
+      </c>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="n">
         <v>202605</v>
       </c>
       <c r="F73" s="1" t="n">
-        <v>15.31</v>
+        <v>3.9</v>
       </c>
       <c r="G73" s="1" t="n">
-        <v>6.62</v>
+        <v>0.78</v>
       </c>
     </row>
     <row r="74">
@@ -22918,7 +22879,7 @@
       <c r="B74" t="inlineStr"/>
       <c r="C74" t="inlineStr">
         <is>
-          <t>DIRECIONADO</t>
+          <t>LIVRE</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
@@ -22926,10 +22887,10 @@
         <v>202605</v>
       </c>
       <c r="F74" s="1" t="n">
-        <v>3.9</v>
+        <v>25.11</v>
       </c>
       <c r="G74" s="1" t="n">
-        <v>0.78</v>
+        <v>10.08</v>
       </c>
     </row>
     <row r="75">
@@ -22938,21 +22899,21 @@
           <t>SPREAD_ICC</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr"/>
-      <c r="C75" t="inlineStr">
-        <is>
-          <t>LIVRE</t>
-        </is>
-      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>PF</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr"/>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="n">
         <v>202605</v>
       </c>
       <c r="F75" s="1" t="n">
-        <v>25.11</v>
+        <v>20.36</v>
       </c>
       <c r="G75" s="1" t="n">
-        <v>10.08</v>
+        <v>6.54</v>
       </c>
     </row>
     <row r="76">
@@ -22966,16 +22927,20 @@
           <t>PF</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr"/>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>DIRECIONADO</t>
+        </is>
+      </c>
       <c r="D76" t="inlineStr"/>
       <c r="E76" t="n">
         <v>202605</v>
       </c>
       <c r="F76" s="1" t="n">
-        <v>20.36</v>
+        <v>4.35</v>
       </c>
       <c r="G76" s="1" t="n">
-        <v>6.54</v>
+        <v>0.93</v>
       </c>
     </row>
     <row r="77">
@@ -22991,7 +22956,7 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>DIRECIONADO</t>
+          <t>LIVRE</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -22999,10 +22964,10 @@
         <v>202605</v>
       </c>
       <c r="F77" s="1" t="n">
-        <v>4.35</v>
+        <v>35.37</v>
       </c>
       <c r="G77" s="1" t="n">
-        <v>0.93</v>
+        <v>7.12</v>
       </c>
     </row>
     <row r="78">
@@ -23013,23 +22978,19 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>PF</t>
-        </is>
-      </c>
-      <c r="C78" t="inlineStr">
-        <is>
-          <t>LIVRE</t>
-        </is>
-      </c>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr"/>
       <c r="D78" t="inlineStr"/>
       <c r="E78" t="n">
         <v>202605</v>
       </c>
       <c r="F78" s="1" t="n">
-        <v>35.37</v>
+        <v>6.98</v>
       </c>
       <c r="G78" s="1" t="n">
-        <v>7.12</v>
+        <v>2.35</v>
       </c>
     </row>
     <row r="79">
@@ -23043,16 +23004,20 @@
           <t>PJ</t>
         </is>
       </c>
-      <c r="C79" t="inlineStr"/>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>DIRECIONADO</t>
+        </is>
+      </c>
       <c r="D79" t="inlineStr"/>
       <c r="E79" t="n">
         <v>202605</v>
       </c>
       <c r="F79" s="1" t="n">
-        <v>6.98</v>
+        <v>3.07</v>
       </c>
       <c r="G79" s="1" t="n">
-        <v>2.35</v>
+        <v>2.33</v>
       </c>
     </row>
     <row r="80">
@@ -23068,7 +23033,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>DIRECIONADO</t>
+          <t>LIVRE</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
@@ -23076,41 +23041,14 @@
         <v>202605</v>
       </c>
       <c r="F80" s="1" t="n">
-        <v>3.07</v>
+        <v>9.890000000000001</v>
       </c>
       <c r="G80" s="1" t="n">
-        <v>2.33</v>
-      </c>
-    </row>
-    <row r="81">
-      <c r="A81" t="inlineStr">
-        <is>
-          <t>SPREAD_ICC</t>
-        </is>
-      </c>
-      <c r="B81" t="inlineStr">
-        <is>
-          <t>PJ</t>
-        </is>
-      </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>LIVRE</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr"/>
-      <c r="E81" t="n">
-        <v>202605</v>
-      </c>
-      <c r="F81" s="1" t="n">
-        <v>9.890000000000001</v>
-      </c>
-      <c r="G81" s="1" t="n">
         <v>7.38</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G81"/>
+  <autoFilter ref="A1:G80"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>